<commit_message>
v0.4.3: HA Reports as six large buttons
Layout sheet updated to match; macro links unchanged.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ribbon-layout.xlsx
+++ b/ribbon-layout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sanat\Downloads\My Excel Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6137FFDE-E637-45EB-902D-C5DEE15E1AB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A0FC02D-3AF7-48A1-8159-33FC712446C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F596BD4C-E1DC-491C-9F85-DFCC71E7EA15}"/>
   </bookViews>
@@ -903,7 +903,7 @@
         <v>16</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>63</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>18</v>
@@ -914,10 +914,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="s">
         <v>19</v>
@@ -926,7 +926,7 @@
         <v>20</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>63</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>21</v>
@@ -983,10 +983,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C6" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" t="s">
         <v>28</v>
@@ -1006,10 +1006,10 @@
         <v>2</v>
       </c>
       <c r="B7" s="6">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C7" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D7" t="s">
         <v>30</v>
@@ -1041,7 +1041,7 @@
         <v>34</v>
       </c>
       <c r="F8" t="s">
-        <v>17</v>
+        <v>63</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>35</v>
@@ -1052,10 +1052,10 @@
         <v>2</v>
       </c>
       <c r="B9" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" t="s">
         <v>36</v>
@@ -1064,7 +1064,7 @@
         <v>37</v>
       </c>
       <c r="F9" t="s">
-        <v>17</v>
+        <v>63</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
v0.4.5: rename group "Retail Formats" to "Buyer Tools"
release.ps1 no longer requires Excel to be closed (the build uses its own
hidden Excel). Layout sheet updated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ribbon-layout.xlsx
+++ b/ribbon-layout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sanat\Downloads\My Excel Tools\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A0FC02D-3AF7-48A1-8159-33FC712446C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9527CA11-09BD-416D-A65E-24CF449F3B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{F596BD4C-E1DC-491C-9F85-DFCC71E7EA15}"/>
   </bookViews>
@@ -50,9 +50,6 @@
     <t>HA Reports</t>
   </si>
   <si>
-    <t>Retail Formats</t>
-  </si>
-  <si>
     <t>Utilities</t>
   </si>
   <si>
@@ -402,6 +399,9 @@
   </si>
   <si>
     <t>grpAbout</t>
+  </si>
+  <si>
+    <t>Buyer Tools</t>
   </si>
 </sst>
 </file>
@@ -865,25 +865,25 @@
   <sheetData>
     <row r="1" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -897,16 +897,16 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>16</v>
-      </c>
       <c r="F2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -920,21 +920,21 @@
         <v>1</v>
       </c>
       <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="F3" t="s">
+        <v>62</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="F3" t="s">
-        <v>63</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="6">
         <v>1</v>
@@ -943,21 +943,21 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>23</v>
-      </c>
-      <c r="F4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="6">
         <v>2</v>
@@ -966,16 +966,16 @@
         <v>1</v>
       </c>
       <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="F5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="F5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -989,16 +989,16 @@
         <v>1</v>
       </c>
       <c r="D6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F6" t="s">
-        <v>63</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -1012,16 +1012,16 @@
         <v>1</v>
       </c>
       <c r="D7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="F7" t="s">
+        <v>62</v>
+      </c>
+      <c r="G7" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="F7" t="s">
-        <v>63</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1035,16 +1035,16 @@
         <v>1</v>
       </c>
       <c r="D8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="F8" t="s">
+        <v>62</v>
+      </c>
+      <c r="G8" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="F8" t="s">
-        <v>63</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1058,21 +1058,21 @@
         <v>1</v>
       </c>
       <c r="D9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="F9" t="s">
+        <v>62</v>
+      </c>
+      <c r="G9" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="F9" t="s">
-        <v>63</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B10" s="6">
         <v>3</v>
@@ -1081,21 +1081,21 @@
         <v>3</v>
       </c>
       <c r="D10" t="s">
+        <v>38</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="F10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" s="4" t="s">
         <v>40</v>
-      </c>
-      <c r="F10" t="s">
-        <v>17</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>3</v>
+        <v>120</v>
       </c>
       <c r="B11" s="6">
         <v>1</v>
@@ -1104,21 +1104,21 @@
         <v>1</v>
       </c>
       <c r="D11" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="F11" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>43</v>
-      </c>
-      <c r="F11" t="s">
-        <v>63</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>3</v>
+        <v>120</v>
       </c>
       <c r="B12" s="6">
         <v>1</v>
@@ -1127,21 +1127,21 @@
         <v>2</v>
       </c>
       <c r="D12" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F12" t="s">
+        <v>62</v>
+      </c>
+      <c r="G12" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="F12" t="s">
-        <v>63</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>3</v>
+        <v>120</v>
       </c>
       <c r="B13" s="6">
         <v>1</v>
@@ -1150,21 +1150,21 @@
         <v>3</v>
       </c>
       <c r="D13" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="F13" t="s">
+        <v>62</v>
+      </c>
+      <c r="G13" s="4" t="s">
         <v>48</v>
-      </c>
-      <c r="F13" t="s">
-        <v>63</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B14" s="6">
         <v>1</v>
@@ -1173,21 +1173,21 @@
         <v>1</v>
       </c>
       <c r="D14" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="F14" t="s">
+        <v>16</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>51</v>
-      </c>
-      <c r="F14" t="s">
-        <v>17</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B15" s="6">
         <v>1</v>
@@ -1196,21 +1196,21 @@
         <v>2</v>
       </c>
       <c r="D15" t="s">
+        <v>52</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F15" t="s">
+        <v>16</v>
+      </c>
+      <c r="G15" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="F15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B16" s="6">
         <v>1</v>
@@ -1219,21 +1219,21 @@
         <v>3</v>
       </c>
       <c r="D16" t="s">
+        <v>54</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="F16" t="s">
-        <v>17</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B17" s="6">
         <v>2</v>
@@ -1242,21 +1242,21 @@
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E17" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F17" t="s">
+        <v>16</v>
+      </c>
+      <c r="G17" s="4" t="s">
         <v>57</v>
-      </c>
-      <c r="F17" t="s">
-        <v>17</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B18" s="6">
         <v>2</v>
@@ -1265,21 +1265,21 @@
         <v>2</v>
       </c>
       <c r="D18" t="s">
+        <v>58</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" s="4" t="s">
         <v>59</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="F18" t="s">
-        <v>17</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B19" s="6">
         <v>1</v>
@@ -1288,21 +1288,21 @@
         <v>1</v>
       </c>
       <c r="D19" t="s">
+        <v>60</v>
+      </c>
+      <c r="E19" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E19" s="5" t="s">
-        <v>62</v>
-      </c>
       <c r="F19" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B20" s="6">
         <v>2</v>
@@ -1311,21 +1311,21 @@
         <v>1</v>
       </c>
       <c r="D20" t="s">
+        <v>64</v>
+      </c>
+      <c r="E20" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="F20" t="s">
+        <v>111</v>
+      </c>
+      <c r="G20" s="4" t="s">
         <v>66</v>
-      </c>
-      <c r="F20" t="s">
-        <v>112</v>
-      </c>
-      <c r="G20" s="4" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B21" s="6">
         <v>3</v>
@@ -1334,21 +1334,21 @@
         <v>1</v>
       </c>
       <c r="D21" t="s">
+        <v>67</v>
+      </c>
+      <c r="E21" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="F21" t="s">
+        <v>111</v>
+      </c>
+      <c r="G21" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="F21" t="s">
-        <v>112</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B22" s="6">
         <v>4</v>
@@ -1357,21 +1357,21 @@
         <v>1</v>
       </c>
       <c r="D22" t="s">
+        <v>70</v>
+      </c>
+      <c r="E22" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="F22" t="s">
+        <v>111</v>
+      </c>
+      <c r="G22" s="4" t="s">
         <v>72</v>
-      </c>
-      <c r="F22" t="s">
-        <v>112</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B23" s="6">
         <v>1</v>
@@ -1380,21 +1380,21 @@
         <v>1</v>
       </c>
       <c r="D23" t="s">
+        <v>73</v>
+      </c>
+      <c r="E23" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="F23" t="s">
+        <v>16</v>
+      </c>
+      <c r="G23" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="F23" t="s">
-        <v>17</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B24" s="6">
         <v>1</v>
@@ -1403,21 +1403,21 @@
         <v>2</v>
       </c>
       <c r="D24" t="s">
+        <v>76</v>
+      </c>
+      <c r="E24" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="F24" t="s">
+        <v>16</v>
+      </c>
+      <c r="G24" s="4" t="s">
         <v>78</v>
-      </c>
-      <c r="F24" t="s">
-        <v>17</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B25" s="6">
         <v>1</v>
@@ -1426,21 +1426,21 @@
         <v>3</v>
       </c>
       <c r="D25" t="s">
+        <v>79</v>
+      </c>
+      <c r="E25" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="F25" t="s">
+        <v>16</v>
+      </c>
+      <c r="G25" s="4" t="s">
         <v>81</v>
-      </c>
-      <c r="F25" t="s">
-        <v>17</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B26" s="6">
         <v>2</v>
@@ -1449,21 +1449,21 @@
         <v>1</v>
       </c>
       <c r="D26" t="s">
+        <v>82</v>
+      </c>
+      <c r="E26" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="F26" t="s">
+        <v>16</v>
+      </c>
+      <c r="G26" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="F26" t="s">
-        <v>17</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B27" s="6">
         <v>2</v>
@@ -1472,21 +1472,21 @@
         <v>2</v>
       </c>
       <c r="D27" t="s">
+        <v>85</v>
+      </c>
+      <c r="E27" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="E27" s="5" t="s">
+      <c r="F27" t="s">
+        <v>16</v>
+      </c>
+      <c r="G27" s="4" t="s">
         <v>87</v>
-      </c>
-      <c r="F27" t="s">
-        <v>17</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B28" s="6">
         <v>2</v>
@@ -1495,21 +1495,21 @@
         <v>3</v>
       </c>
       <c r="D28" t="s">
+        <v>88</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="F28" t="s">
+        <v>16</v>
+      </c>
+      <c r="G28" s="4" t="s">
         <v>89</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="F28" t="s">
-        <v>17</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B29" s="6">
         <v>1</v>
@@ -1518,19 +1518,19 @@
         <v>1</v>
       </c>
       <c r="D29" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E29" s="5"/>
       <c r="F29" t="s">
+        <v>91</v>
+      </c>
+      <c r="G29" s="4" t="s">
         <v>92</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B30" s="6">
         <v>1</v>
@@ -1539,19 +1539,19 @@
         <v>2</v>
       </c>
       <c r="D30" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E30" s="5"/>
       <c r="F30" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B31" s="6">
         <v>1</v>
@@ -1560,14 +1560,14 @@
         <v>3</v>
       </c>
       <c r="D31" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E31" s="5"/>
       <c r="F31" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1684,10 +1684,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -1698,62 +1698,62 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>120</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6">
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7">
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -1771,67 +1771,67 @@
   <sheetData>
     <row r="1" spans="1:1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>